<commit_message>
Permitir Colegio/Curso/Letra en la planilla de correccion (una vez por archivo)
</commit_message>
<xml_diff>
--- a/assets/Planilla_de_correccion.xlsx
+++ b/assets/Planilla_de_correccion.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="600" windowWidth="33600" windowHeight="19140" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Correccion" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -25,46 +26,35 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF402A63"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FF333333"/>
+      <color rgb="00402A63"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="00402A63"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00402A63"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FF0000FF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
       <b val="1"/>
-      <color rgb="FF000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color rgb="FF0000FF"/>
-      <sz val="10"/>
+      <color rgb="00402A63"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,17 +63,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF5B3B8C"/>
+        <fgColor rgb="005B3B8C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF402A63"/>
+        <fgColor rgb="00F5F2FB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF8E8"/>
+        <fgColor rgb="00E1D9F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF8E8"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,54 +92,45 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="00C9BEDD"/>
       </left>
       <right style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="00C9BEDD"/>
       </right>
       <top style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="00C9BEDD"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFCCCCCC"/>
+        <color rgb="00C9BEDD"/>
       </bottom>
-      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -216,21 +202,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>UMAG</author>
-  </authors>
-  <commentList>
-    <comment ref="C5" authorId="0" shapeId="0">
-      <text>
-        <t>Columnas 1 a 24 = ítems del cuestionario, en el mismo orden que la hoja de aplicación en papel.</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -522,327 +493,327 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:AF47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="11" min="1" max="1"/>
-    <col width="16" customWidth="1" style="11" min="2" max="2"/>
-    <col width="4.5" customWidth="1" style="11" min="3" max="26"/>
-    <col width="15" customWidth="1" style="11" min="27" max="32"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="4.5" customWidth="1" min="3" max="3"/>
+    <col width="4.5" customWidth="1" min="4" max="4"/>
+    <col width="4.5" customWidth="1" min="5" max="5"/>
+    <col width="4.5" customWidth="1" min="6" max="6"/>
+    <col width="4.5" customWidth="1" min="7" max="7"/>
+    <col width="4.5" customWidth="1" min="8" max="8"/>
+    <col width="4.5" customWidth="1" min="9" max="9"/>
+    <col width="4.5" customWidth="1" min="10" max="10"/>
+    <col width="4.5" customWidth="1" min="11" max="11"/>
+    <col width="4.5" customWidth="1" min="12" max="12"/>
+    <col width="4.5" customWidth="1" min="13" max="13"/>
+    <col width="4.5" customWidth="1" min="14" max="14"/>
+    <col width="4.5" customWidth="1" min="15" max="15"/>
+    <col width="4.5" customWidth="1" min="16" max="16"/>
+    <col width="4.5" customWidth="1" min="17" max="17"/>
+    <col width="4.5" customWidth="1" min="18" max="18"/>
+    <col width="4.5" customWidth="1" min="19" max="19"/>
+    <col width="4.5" customWidth="1" min="20" max="20"/>
+    <col width="4.5" customWidth="1" min="21" max="21"/>
+    <col width="4.5" customWidth="1" min="22" max="22"/>
+    <col width="4.5" customWidth="1" min="23" max="23"/>
+    <col width="4.5" customWidth="1" min="24" max="24"/>
+    <col width="4.5" customWidth="1" min="25" max="25"/>
+    <col width="4.5" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="13" customWidth="1" min="29" max="29"/>
+    <col width="13" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1" s="11">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Planilla de corrección — Orientando mis Intereses (8° Básico)</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="48" customHeight="1" s="11">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>Completa una fila por estudiante: Nombre, RUT y las 24 respuestas en el mismo orden en que aparecen en la hoja de aplicación en papel (3 = Me gusta/Me interesa · 2 = No sé · 1 = No me gusta/No me interesa). Las columnas de área (fondo gris, en negrita) se calculan solas — no las edites. El colegio, curso, letra y fecha de aplicación NO van en esta planilla: se asignan en la aplicación web al momento de subir este archivo (así no hay que repetirlos por estudiante). Cuando termines, sube este mismo archivo .xlsx directamente en la app, en la pestaña "Ingresar datos".</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="5" ht="30" customHeight="1" s="11">
-      <c r="A5" s="1" t="inlineStr">
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Completa una fila por estudiante: Nombre, RUT (opcional — muchos estudiantes de esta edad no lo saben de memoria) y las 24 respuestas en el mismo orden en que aparecen en la hoja de aplicación en papel (3 = Me gusta/Me interesa · 2 = No sé · 1 = No me gusta/No me interesa). Las columnas de área (fondo gris, en negrita) se calculan solas — no las edites. Completa Colegio, Curso y Letra UNA SOLA VEZ en los campos de abajo: valen para todos los estudiantes de este archivo (cada planilla es siempre un curso de un colegio). Cuando termines, sube este mismo archivo .xlsx directamente en la app, en la pestaña "Ingresar datos".</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="46" customHeight="1"/>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Colegio:</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
+      <c r="E4" s="4" t="n"/>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Curso:</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n"/>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Letra:</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="n"/>
+    </row>
+    <row r="5" ht="6" customHeight="1"/>
+    <row r="6" ht="32" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Nombre</t>
         </is>
       </c>
-      <c r="B5" s="1" t="inlineStr">
+      <c r="B6" s="5" t="inlineStr">
         <is>
           <t>RUT</t>
         </is>
       </c>
-      <c r="C5" s="1" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" s="1" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E5" s="1" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="F5" s="1" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="G5" s="1" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="H5" s="1" t="inlineStr">
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="I5" s="1" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="J5" s="1" t="inlineStr">
+      <c r="J6" s="6" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="K5" s="1" t="inlineStr">
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="L5" s="1" t="inlineStr">
+      <c r="L6" s="6" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="M5" s="1" t="inlineStr">
+      <c r="M6" s="6" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="N5" s="1" t="inlineStr">
+      <c r="N6" s="6" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="O5" s="1" t="inlineStr">
+      <c r="O6" s="6" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="P5" s="1" t="inlineStr">
+      <c r="P6" s="6" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="Q5" s="1" t="inlineStr">
+      <c r="Q6" s="6" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="R5" s="1" t="inlineStr">
+      <c r="R6" s="6" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="S5" s="1" t="inlineStr">
+      <c r="S6" s="6" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="T5" s="1" t="inlineStr">
+      <c r="T6" s="6" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="U5" s="1" t="inlineStr">
+      <c r="U6" s="6" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="V5" s="1" t="inlineStr">
+      <c r="V6" s="6" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="W5" s="1" t="inlineStr">
+      <c r="W6" s="6" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="X5" s="1" t="inlineStr">
+      <c r="X6" s="6" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="Y5" s="1" t="inlineStr">
+      <c r="Y6" s="6" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="Z5" s="1" t="inlineStr">
+      <c r="Z6" s="6" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="AA5" s="2" t="inlineStr">
+      <c r="AA6" s="7" t="inlineStr">
         <is>
           <t>Ciencias</t>
         </is>
       </c>
-      <c r="AB5" s="2" t="inlineStr">
+      <c r="AB6" s="7" t="inlineStr">
         <is>
           <t>Humanidades y Ciencias Sociales</t>
         </is>
       </c>
-      <c r="AC5" s="2" t="inlineStr">
+      <c r="AC6" s="7" t="inlineStr">
         <is>
           <t>Artístico-Expresivo</t>
         </is>
       </c>
-      <c r="AD5" s="2" t="inlineStr">
+      <c r="AD6" s="7" t="inlineStr">
         <is>
           <t>Técnico-Manual</t>
         </is>
       </c>
-      <c r="AE5" s="2" t="inlineStr">
+      <c r="AE6" s="7" t="inlineStr">
         <is>
           <t>Salud y Cuidado</t>
         </is>
       </c>
-      <c r="AF5" s="2" t="inlineStr">
+      <c r="AF6" s="7" t="inlineStr">
         <is>
           <t>Administración y Negocios</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Ejemplo: Ana Pérez</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>21.345.678-9</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C7" t="n">
         <v>3</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D7" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E7" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F7" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G7" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="4" t="n">
+      <c r="H7" t="n">
         <v>3</v>
       </c>
-      <c r="I6" s="4" t="n">
+      <c r="I7" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="4" t="n">
+      <c r="J7" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="4" t="n">
+      <c r="K7" t="n">
         <v>2</v>
       </c>
-      <c r="L6" s="4" t="n">
+      <c r="L7" t="n">
         <v>3</v>
       </c>
-      <c r="M6" s="4" t="n">
+      <c r="M7" t="n">
         <v>3</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N7" t="n">
         <v>2</v>
       </c>
-      <c r="O6" s="4" t="n">
+      <c r="O7" t="n">
         <v>2</v>
       </c>
-      <c r="P6" s="4" t="n">
+      <c r="P7" t="n">
         <v>3</v>
       </c>
-      <c r="Q6" s="4" t="n">
+      <c r="Q7" t="n">
         <v>1</v>
       </c>
-      <c r="R6" s="4" t="n">
+      <c r="R7" t="n">
         <v>2</v>
       </c>
-      <c r="S6" s="4" t="n">
+      <c r="S7" t="n">
         <v>3</v>
       </c>
-      <c r="T6" s="4" t="n">
+      <c r="T7" t="n">
         <v>3</v>
       </c>
-      <c r="U6" s="4" t="n">
+      <c r="U7" t="n">
         <v>3</v>
       </c>
-      <c r="V6" s="4" t="n">
+      <c r="V7" t="n">
         <v>2</v>
       </c>
-      <c r="W6" s="4" t="n">
+      <c r="W7" t="n">
         <v>3</v>
       </c>
-      <c r="X6" s="4" t="n">
+      <c r="X7" t="n">
         <v>1</v>
       </c>
-      <c r="Y6" s="4" t="n">
+      <c r="Y7" t="n">
         <v>2</v>
       </c>
-      <c r="Z6" s="4" t="n">
+      <c r="Z7" t="n">
         <v>3</v>
       </c>
-      <c r="AA6" s="5">
-        <f>SUM(C6,I6,O6,U6)-4</f>
-        <v/>
-      </c>
-      <c r="AB6" s="5">
-        <f>SUM(D6,J6,P6,V6)-4</f>
-        <v/>
-      </c>
-      <c r="AC6" s="5">
-        <f>SUM(E6,K6,Q6,W6)-4</f>
-        <v/>
-      </c>
-      <c r="AD6" s="5">
-        <f>SUM(F6,L6,R6,X6)-4</f>
-        <v/>
-      </c>
-      <c r="AE6" s="5">
-        <f>SUM(G6,M6,S6,Y6)-4</f>
-        <v/>
-      </c>
-      <c r="AF6" s="5">
-        <f>SUM(H6,N6,T6,Z6)-4</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="n"/>
-      <c r="B7" s="9" t="n"/>
-      <c r="C7" s="7" t="n"/>
-      <c r="D7" s="7" t="n"/>
-      <c r="E7" s="7" t="n"/>
-      <c r="F7" s="7" t="n"/>
-      <c r="G7" s="7" t="n"/>
-      <c r="H7" s="7" t="n"/>
-      <c r="I7" s="7" t="n"/>
-      <c r="J7" s="7" t="n"/>
-      <c r="K7" s="7" t="n"/>
-      <c r="L7" s="7" t="n"/>
-      <c r="M7" s="7" t="n"/>
-      <c r="N7" s="7" t="n"/>
-      <c r="O7" s="7" t="n"/>
-      <c r="P7" s="7" t="n"/>
-      <c r="Q7" s="7" t="n"/>
-      <c r="R7" s="7" t="n"/>
-      <c r="S7" s="7" t="n"/>
-      <c r="T7" s="7" t="n"/>
-      <c r="U7" s="7" t="n"/>
-      <c r="V7" s="7" t="n"/>
-      <c r="W7" s="7" t="n"/>
-      <c r="X7" s="7" t="n"/>
-      <c r="Y7" s="7" t="n"/>
-      <c r="Z7" s="7" t="n"/>
       <c r="AA7" s="8">
         <f>SUM(C7,I7,O7,U7)-4</f>
         <v/>
@@ -869,32 +840,6 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n"/>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="7" t="n"/>
-      <c r="E8" s="7" t="n"/>
-      <c r="F8" s="7" t="n"/>
-      <c r="G8" s="7" t="n"/>
-      <c r="H8" s="7" t="n"/>
-      <c r="I8" s="7" t="n"/>
-      <c r="J8" s="7" t="n"/>
-      <c r="K8" s="7" t="n"/>
-      <c r="L8" s="7" t="n"/>
-      <c r="M8" s="7" t="n"/>
-      <c r="N8" s="7" t="n"/>
-      <c r="O8" s="7" t="n"/>
-      <c r="P8" s="7" t="n"/>
-      <c r="Q8" s="7" t="n"/>
-      <c r="R8" s="7" t="n"/>
-      <c r="S8" s="7" t="n"/>
-      <c r="T8" s="7" t="n"/>
-      <c r="U8" s="7" t="n"/>
-      <c r="V8" s="7" t="n"/>
-      <c r="W8" s="7" t="n"/>
-      <c r="X8" s="7" t="n"/>
-      <c r="Y8" s="7" t="n"/>
-      <c r="Z8" s="7" t="n"/>
       <c r="AA8" s="8">
         <f>SUM(C8,I8,O8,U8)-4</f>
         <v/>
@@ -921,32 +866,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n"/>
-      <c r="B9" s="9" t="n"/>
-      <c r="C9" s="7" t="n"/>
-      <c r="D9" s="7" t="n"/>
-      <c r="E9" s="7" t="n"/>
-      <c r="F9" s="7" t="n"/>
-      <c r="G9" s="7" t="n"/>
-      <c r="H9" s="7" t="n"/>
-      <c r="I9" s="7" t="n"/>
-      <c r="J9" s="7" t="n"/>
-      <c r="K9" s="7" t="n"/>
-      <c r="L9" s="7" t="n"/>
-      <c r="M9" s="7" t="n"/>
-      <c r="N9" s="7" t="n"/>
-      <c r="O9" s="7" t="n"/>
-      <c r="P9" s="7" t="n"/>
-      <c r="Q9" s="7" t="n"/>
-      <c r="R9" s="7" t="n"/>
-      <c r="S9" s="7" t="n"/>
-      <c r="T9" s="7" t="n"/>
-      <c r="U9" s="7" t="n"/>
-      <c r="V9" s="7" t="n"/>
-      <c r="W9" s="7" t="n"/>
-      <c r="X9" s="7" t="n"/>
-      <c r="Y9" s="7" t="n"/>
-      <c r="Z9" s="7" t="n"/>
       <c r="AA9" s="8">
         <f>SUM(C9,I9,O9,U9)-4</f>
         <v/>
@@ -973,32 +892,6 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="7" t="n"/>
-      <c r="D10" s="7" t="n"/>
-      <c r="E10" s="7" t="n"/>
-      <c r="F10" s="7" t="n"/>
-      <c r="G10" s="7" t="n"/>
-      <c r="H10" s="7" t="n"/>
-      <c r="I10" s="7" t="n"/>
-      <c r="J10" s="7" t="n"/>
-      <c r="K10" s="7" t="n"/>
-      <c r="L10" s="7" t="n"/>
-      <c r="M10" s="7" t="n"/>
-      <c r="N10" s="7" t="n"/>
-      <c r="O10" s="7" t="n"/>
-      <c r="P10" s="7" t="n"/>
-      <c r="Q10" s="7" t="n"/>
-      <c r="R10" s="7" t="n"/>
-      <c r="S10" s="7" t="n"/>
-      <c r="T10" s="7" t="n"/>
-      <c r="U10" s="7" t="n"/>
-      <c r="V10" s="7" t="n"/>
-      <c r="W10" s="7" t="n"/>
-      <c r="X10" s="7" t="n"/>
-      <c r="Y10" s="7" t="n"/>
-      <c r="Z10" s="7" t="n"/>
       <c r="AA10" s="8">
         <f>SUM(C10,I10,O10,U10)-4</f>
         <v/>
@@ -1025,32 +918,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n"/>
-      <c r="B11" s="9" t="n"/>
-      <c r="C11" s="7" t="n"/>
-      <c r="D11" s="7" t="n"/>
-      <c r="E11" s="7" t="n"/>
-      <c r="F11" s="7" t="n"/>
-      <c r="G11" s="7" t="n"/>
-      <c r="H11" s="7" t="n"/>
-      <c r="I11" s="7" t="n"/>
-      <c r="J11" s="7" t="n"/>
-      <c r="K11" s="7" t="n"/>
-      <c r="L11" s="7" t="n"/>
-      <c r="M11" s="7" t="n"/>
-      <c r="N11" s="7" t="n"/>
-      <c r="O11" s="7" t="n"/>
-      <c r="P11" s="7" t="n"/>
-      <c r="Q11" s="7" t="n"/>
-      <c r="R11" s="7" t="n"/>
-      <c r="S11" s="7" t="n"/>
-      <c r="T11" s="7" t="n"/>
-      <c r="U11" s="7" t="n"/>
-      <c r="V11" s="7" t="n"/>
-      <c r="W11" s="7" t="n"/>
-      <c r="X11" s="7" t="n"/>
-      <c r="Y11" s="7" t="n"/>
-      <c r="Z11" s="7" t="n"/>
       <c r="AA11" s="8">
         <f>SUM(C11,I11,O11,U11)-4</f>
         <v/>
@@ -1077,32 +944,6 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="7" t="n"/>
-      <c r="D12" s="7" t="n"/>
-      <c r="E12" s="7" t="n"/>
-      <c r="F12" s="7" t="n"/>
-      <c r="G12" s="7" t="n"/>
-      <c r="H12" s="7" t="n"/>
-      <c r="I12" s="7" t="n"/>
-      <c r="J12" s="7" t="n"/>
-      <c r="K12" s="7" t="n"/>
-      <c r="L12" s="7" t="n"/>
-      <c r="M12" s="7" t="n"/>
-      <c r="N12" s="7" t="n"/>
-      <c r="O12" s="7" t="n"/>
-      <c r="P12" s="7" t="n"/>
-      <c r="Q12" s="7" t="n"/>
-      <c r="R12" s="7" t="n"/>
-      <c r="S12" s="7" t="n"/>
-      <c r="T12" s="7" t="n"/>
-      <c r="U12" s="7" t="n"/>
-      <c r="V12" s="7" t="n"/>
-      <c r="W12" s="7" t="n"/>
-      <c r="X12" s="7" t="n"/>
-      <c r="Y12" s="7" t="n"/>
-      <c r="Z12" s="7" t="n"/>
       <c r="AA12" s="8">
         <f>SUM(C12,I12,O12,U12)-4</f>
         <v/>
@@ -1129,32 +970,6 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="7" t="n"/>
-      <c r="D13" s="7" t="n"/>
-      <c r="E13" s="7" t="n"/>
-      <c r="F13" s="7" t="n"/>
-      <c r="G13" s="7" t="n"/>
-      <c r="H13" s="7" t="n"/>
-      <c r="I13" s="7" t="n"/>
-      <c r="J13" s="7" t="n"/>
-      <c r="K13" s="7" t="n"/>
-      <c r="L13" s="7" t="n"/>
-      <c r="M13" s="7" t="n"/>
-      <c r="N13" s="7" t="n"/>
-      <c r="O13" s="7" t="n"/>
-      <c r="P13" s="7" t="n"/>
-      <c r="Q13" s="7" t="n"/>
-      <c r="R13" s="7" t="n"/>
-      <c r="S13" s="7" t="n"/>
-      <c r="T13" s="7" t="n"/>
-      <c r="U13" s="7" t="n"/>
-      <c r="V13" s="7" t="n"/>
-      <c r="W13" s="7" t="n"/>
-      <c r="X13" s="7" t="n"/>
-      <c r="Y13" s="7" t="n"/>
-      <c r="Z13" s="7" t="n"/>
       <c r="AA13" s="8">
         <f>SUM(C13,I13,O13,U13)-4</f>
         <v/>
@@ -1181,32 +996,6 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="7" t="n"/>
-      <c r="D14" s="7" t="n"/>
-      <c r="E14" s="7" t="n"/>
-      <c r="F14" s="7" t="n"/>
-      <c r="G14" s="7" t="n"/>
-      <c r="H14" s="7" t="n"/>
-      <c r="I14" s="7" t="n"/>
-      <c r="J14" s="7" t="n"/>
-      <c r="K14" s="7" t="n"/>
-      <c r="L14" s="7" t="n"/>
-      <c r="M14" s="7" t="n"/>
-      <c r="N14" s="7" t="n"/>
-      <c r="O14" s="7" t="n"/>
-      <c r="P14" s="7" t="n"/>
-      <c r="Q14" s="7" t="n"/>
-      <c r="R14" s="7" t="n"/>
-      <c r="S14" s="7" t="n"/>
-      <c r="T14" s="7" t="n"/>
-      <c r="U14" s="7" t="n"/>
-      <c r="V14" s="7" t="n"/>
-      <c r="W14" s="7" t="n"/>
-      <c r="X14" s="7" t="n"/>
-      <c r="Y14" s="7" t="n"/>
-      <c r="Z14" s="7" t="n"/>
       <c r="AA14" s="8">
         <f>SUM(C14,I14,O14,U14)-4</f>
         <v/>
@@ -1233,32 +1022,6 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="6" t="n"/>
-      <c r="B15" s="6" t="n"/>
-      <c r="C15" s="7" t="n"/>
-      <c r="D15" s="7" t="n"/>
-      <c r="E15" s="7" t="n"/>
-      <c r="F15" s="7" t="n"/>
-      <c r="G15" s="7" t="n"/>
-      <c r="H15" s="7" t="n"/>
-      <c r="I15" s="7" t="n"/>
-      <c r="J15" s="7" t="n"/>
-      <c r="K15" s="7" t="n"/>
-      <c r="L15" s="7" t="n"/>
-      <c r="M15" s="7" t="n"/>
-      <c r="N15" s="7" t="n"/>
-      <c r="O15" s="7" t="n"/>
-      <c r="P15" s="7" t="n"/>
-      <c r="Q15" s="7" t="n"/>
-      <c r="R15" s="7" t="n"/>
-      <c r="S15" s="7" t="n"/>
-      <c r="T15" s="7" t="n"/>
-      <c r="U15" s="7" t="n"/>
-      <c r="V15" s="7" t="n"/>
-      <c r="W15" s="7" t="n"/>
-      <c r="X15" s="7" t="n"/>
-      <c r="Y15" s="7" t="n"/>
-      <c r="Z15" s="7" t="n"/>
       <c r="AA15" s="8">
         <f>SUM(C15,I15,O15,U15)-4</f>
         <v/>
@@ -1285,32 +1048,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6" t="n"/>
-      <c r="C16" s="7" t="n"/>
-      <c r="D16" s="7" t="n"/>
-      <c r="E16" s="7" t="n"/>
-      <c r="F16" s="7" t="n"/>
-      <c r="G16" s="7" t="n"/>
-      <c r="H16" s="7" t="n"/>
-      <c r="I16" s="7" t="n"/>
-      <c r="J16" s="7" t="n"/>
-      <c r="K16" s="7" t="n"/>
-      <c r="L16" s="7" t="n"/>
-      <c r="M16" s="7" t="n"/>
-      <c r="N16" s="7" t="n"/>
-      <c r="O16" s="7" t="n"/>
-      <c r="P16" s="7" t="n"/>
-      <c r="Q16" s="7" t="n"/>
-      <c r="R16" s="7" t="n"/>
-      <c r="S16" s="7" t="n"/>
-      <c r="T16" s="7" t="n"/>
-      <c r="U16" s="7" t="n"/>
-      <c r="V16" s="7" t="n"/>
-      <c r="W16" s="7" t="n"/>
-      <c r="X16" s="7" t="n"/>
-      <c r="Y16" s="7" t="n"/>
-      <c r="Z16" s="7" t="n"/>
       <c r="AA16" s="8">
         <f>SUM(C16,I16,O16,U16)-4</f>
         <v/>
@@ -1337,32 +1074,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="6" t="n"/>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="7" t="n"/>
-      <c r="D17" s="7" t="n"/>
-      <c r="E17" s="7" t="n"/>
-      <c r="F17" s="7" t="n"/>
-      <c r="G17" s="7" t="n"/>
-      <c r="H17" s="7" t="n"/>
-      <c r="I17" s="7" t="n"/>
-      <c r="J17" s="7" t="n"/>
-      <c r="K17" s="7" t="n"/>
-      <c r="L17" s="7" t="n"/>
-      <c r="M17" s="7" t="n"/>
-      <c r="N17" s="7" t="n"/>
-      <c r="O17" s="7" t="n"/>
-      <c r="P17" s="7" t="n"/>
-      <c r="Q17" s="7" t="n"/>
-      <c r="R17" s="7" t="n"/>
-      <c r="S17" s="7" t="n"/>
-      <c r="T17" s="7" t="n"/>
-      <c r="U17" s="7" t="n"/>
-      <c r="V17" s="7" t="n"/>
-      <c r="W17" s="7" t="n"/>
-      <c r="X17" s="7" t="n"/>
-      <c r="Y17" s="7" t="n"/>
-      <c r="Z17" s="7" t="n"/>
       <c r="AA17" s="8">
         <f>SUM(C17,I17,O17,U17)-4</f>
         <v/>
@@ -1389,32 +1100,6 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="n"/>
-      <c r="C18" s="7" t="n"/>
-      <c r="D18" s="7" t="n"/>
-      <c r="E18" s="7" t="n"/>
-      <c r="F18" s="7" t="n"/>
-      <c r="G18" s="7" t="n"/>
-      <c r="H18" s="7" t="n"/>
-      <c r="I18" s="7" t="n"/>
-      <c r="J18" s="7" t="n"/>
-      <c r="K18" s="7" t="n"/>
-      <c r="L18" s="7" t="n"/>
-      <c r="M18" s="7" t="n"/>
-      <c r="N18" s="7" t="n"/>
-      <c r="O18" s="7" t="n"/>
-      <c r="P18" s="7" t="n"/>
-      <c r="Q18" s="7" t="n"/>
-      <c r="R18" s="7" t="n"/>
-      <c r="S18" s="7" t="n"/>
-      <c r="T18" s="7" t="n"/>
-      <c r="U18" s="7" t="n"/>
-      <c r="V18" s="7" t="n"/>
-      <c r="W18" s="7" t="n"/>
-      <c r="X18" s="7" t="n"/>
-      <c r="Y18" s="7" t="n"/>
-      <c r="Z18" s="7" t="n"/>
       <c r="AA18" s="8">
         <f>SUM(C18,I18,O18,U18)-4</f>
         <v/>
@@ -1441,32 +1126,6 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="n"/>
-      <c r="B19" s="6" t="n"/>
-      <c r="C19" s="7" t="n"/>
-      <c r="D19" s="7" t="n"/>
-      <c r="E19" s="7" t="n"/>
-      <c r="F19" s="7" t="n"/>
-      <c r="G19" s="7" t="n"/>
-      <c r="H19" s="7" t="n"/>
-      <c r="I19" s="7" t="n"/>
-      <c r="J19" s="7" t="n"/>
-      <c r="K19" s="7" t="n"/>
-      <c r="L19" s="7" t="n"/>
-      <c r="M19" s="7" t="n"/>
-      <c r="N19" s="7" t="n"/>
-      <c r="O19" s="7" t="n"/>
-      <c r="P19" s="7" t="n"/>
-      <c r="Q19" s="7" t="n"/>
-      <c r="R19" s="7" t="n"/>
-      <c r="S19" s="7" t="n"/>
-      <c r="T19" s="7" t="n"/>
-      <c r="U19" s="7" t="n"/>
-      <c r="V19" s="7" t="n"/>
-      <c r="W19" s="7" t="n"/>
-      <c r="X19" s="7" t="n"/>
-      <c r="Y19" s="7" t="n"/>
-      <c r="Z19" s="7" t="n"/>
       <c r="AA19" s="8">
         <f>SUM(C19,I19,O19,U19)-4</f>
         <v/>
@@ -1493,32 +1152,6 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="7" t="n"/>
-      <c r="D20" s="7" t="n"/>
-      <c r="E20" s="7" t="n"/>
-      <c r="F20" s="7" t="n"/>
-      <c r="G20" s="7" t="n"/>
-      <c r="H20" s="7" t="n"/>
-      <c r="I20" s="7" t="n"/>
-      <c r="J20" s="7" t="n"/>
-      <c r="K20" s="7" t="n"/>
-      <c r="L20" s="7" t="n"/>
-      <c r="M20" s="7" t="n"/>
-      <c r="N20" s="7" t="n"/>
-      <c r="O20" s="7" t="n"/>
-      <c r="P20" s="7" t="n"/>
-      <c r="Q20" s="7" t="n"/>
-      <c r="R20" s="7" t="n"/>
-      <c r="S20" s="7" t="n"/>
-      <c r="T20" s="7" t="n"/>
-      <c r="U20" s="7" t="n"/>
-      <c r="V20" s="7" t="n"/>
-      <c r="W20" s="7" t="n"/>
-      <c r="X20" s="7" t="n"/>
-      <c r="Y20" s="7" t="n"/>
-      <c r="Z20" s="7" t="n"/>
       <c r="AA20" s="8">
         <f>SUM(C20,I20,O20,U20)-4</f>
         <v/>
@@ -1545,32 +1178,6 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="6" t="n"/>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="7" t="n"/>
-      <c r="D21" s="7" t="n"/>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="7" t="n"/>
-      <c r="G21" s="7" t="n"/>
-      <c r="H21" s="7" t="n"/>
-      <c r="I21" s="7" t="n"/>
-      <c r="J21" s="7" t="n"/>
-      <c r="K21" s="7" t="n"/>
-      <c r="L21" s="7" t="n"/>
-      <c r="M21" s="7" t="n"/>
-      <c r="N21" s="7" t="n"/>
-      <c r="O21" s="7" t="n"/>
-      <c r="P21" s="7" t="n"/>
-      <c r="Q21" s="7" t="n"/>
-      <c r="R21" s="7" t="n"/>
-      <c r="S21" s="7" t="n"/>
-      <c r="T21" s="7" t="n"/>
-      <c r="U21" s="7" t="n"/>
-      <c r="V21" s="7" t="n"/>
-      <c r="W21" s="7" t="n"/>
-      <c r="X21" s="7" t="n"/>
-      <c r="Y21" s="7" t="n"/>
-      <c r="Z21" s="7" t="n"/>
       <c r="AA21" s="8">
         <f>SUM(C21,I21,O21,U21)-4</f>
         <v/>
@@ -1597,32 +1204,6 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="7" t="n"/>
-      <c r="D22" s="7" t="n"/>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="7" t="n"/>
-      <c r="G22" s="7" t="n"/>
-      <c r="H22" s="7" t="n"/>
-      <c r="I22" s="7" t="n"/>
-      <c r="J22" s="7" t="n"/>
-      <c r="K22" s="7" t="n"/>
-      <c r="L22" s="7" t="n"/>
-      <c r="M22" s="7" t="n"/>
-      <c r="N22" s="7" t="n"/>
-      <c r="O22" s="7" t="n"/>
-      <c r="P22" s="7" t="n"/>
-      <c r="Q22" s="7" t="n"/>
-      <c r="R22" s="7" t="n"/>
-      <c r="S22" s="7" t="n"/>
-      <c r="T22" s="7" t="n"/>
-      <c r="U22" s="7" t="n"/>
-      <c r="V22" s="7" t="n"/>
-      <c r="W22" s="7" t="n"/>
-      <c r="X22" s="7" t="n"/>
-      <c r="Y22" s="7" t="n"/>
-      <c r="Z22" s="7" t="n"/>
       <c r="AA22" s="8">
         <f>SUM(C22,I22,O22,U22)-4</f>
         <v/>
@@ -1649,32 +1230,6 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="6" t="n"/>
-      <c r="B23" s="6" t="n"/>
-      <c r="C23" s="7" t="n"/>
-      <c r="D23" s="7" t="n"/>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="7" t="n"/>
-      <c r="G23" s="7" t="n"/>
-      <c r="H23" s="7" t="n"/>
-      <c r="I23" s="7" t="n"/>
-      <c r="J23" s="7" t="n"/>
-      <c r="K23" s="7" t="n"/>
-      <c r="L23" s="7" t="n"/>
-      <c r="M23" s="7" t="n"/>
-      <c r="N23" s="7" t="n"/>
-      <c r="O23" s="7" t="n"/>
-      <c r="P23" s="7" t="n"/>
-      <c r="Q23" s="7" t="n"/>
-      <c r="R23" s="7" t="n"/>
-      <c r="S23" s="7" t="n"/>
-      <c r="T23" s="7" t="n"/>
-      <c r="U23" s="7" t="n"/>
-      <c r="V23" s="7" t="n"/>
-      <c r="W23" s="7" t="n"/>
-      <c r="X23" s="7" t="n"/>
-      <c r="Y23" s="7" t="n"/>
-      <c r="Z23" s="7" t="n"/>
       <c r="AA23" s="8">
         <f>SUM(C23,I23,O23,U23)-4</f>
         <v/>
@@ -1701,32 +1256,6 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="n"/>
-      <c r="C24" s="7" t="n"/>
-      <c r="D24" s="7" t="n"/>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="7" t="n"/>
-      <c r="G24" s="7" t="n"/>
-      <c r="H24" s="7" t="n"/>
-      <c r="I24" s="7" t="n"/>
-      <c r="J24" s="7" t="n"/>
-      <c r="K24" s="7" t="n"/>
-      <c r="L24" s="7" t="n"/>
-      <c r="M24" s="7" t="n"/>
-      <c r="N24" s="7" t="n"/>
-      <c r="O24" s="7" t="n"/>
-      <c r="P24" s="7" t="n"/>
-      <c r="Q24" s="7" t="n"/>
-      <c r="R24" s="7" t="n"/>
-      <c r="S24" s="7" t="n"/>
-      <c r="T24" s="7" t="n"/>
-      <c r="U24" s="7" t="n"/>
-      <c r="V24" s="7" t="n"/>
-      <c r="W24" s="7" t="n"/>
-      <c r="X24" s="7" t="n"/>
-      <c r="Y24" s="7" t="n"/>
-      <c r="Z24" s="7" t="n"/>
       <c r="AA24" s="8">
         <f>SUM(C24,I24,O24,U24)-4</f>
         <v/>
@@ -1753,32 +1282,6 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="6" t="n"/>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="7" t="n"/>
-      <c r="D25" s="7" t="n"/>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="7" t="n"/>
-      <c r="G25" s="7" t="n"/>
-      <c r="H25" s="7" t="n"/>
-      <c r="I25" s="7" t="n"/>
-      <c r="J25" s="7" t="n"/>
-      <c r="K25" s="7" t="n"/>
-      <c r="L25" s="7" t="n"/>
-      <c r="M25" s="7" t="n"/>
-      <c r="N25" s="7" t="n"/>
-      <c r="O25" s="7" t="n"/>
-      <c r="P25" s="7" t="n"/>
-      <c r="Q25" s="7" t="n"/>
-      <c r="R25" s="7" t="n"/>
-      <c r="S25" s="7" t="n"/>
-      <c r="T25" s="7" t="n"/>
-      <c r="U25" s="7" t="n"/>
-      <c r="V25" s="7" t="n"/>
-      <c r="W25" s="7" t="n"/>
-      <c r="X25" s="7" t="n"/>
-      <c r="Y25" s="7" t="n"/>
-      <c r="Z25" s="7" t="n"/>
       <c r="AA25" s="8">
         <f>SUM(C25,I25,O25,U25)-4</f>
         <v/>
@@ -1805,32 +1308,6 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="7" t="n"/>
-      <c r="D26" s="7" t="n"/>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="7" t="n"/>
-      <c r="G26" s="7" t="n"/>
-      <c r="H26" s="7" t="n"/>
-      <c r="I26" s="7" t="n"/>
-      <c r="J26" s="7" t="n"/>
-      <c r="K26" s="7" t="n"/>
-      <c r="L26" s="7" t="n"/>
-      <c r="M26" s="7" t="n"/>
-      <c r="N26" s="7" t="n"/>
-      <c r="O26" s="7" t="n"/>
-      <c r="P26" s="7" t="n"/>
-      <c r="Q26" s="7" t="n"/>
-      <c r="R26" s="7" t="n"/>
-      <c r="S26" s="7" t="n"/>
-      <c r="T26" s="7" t="n"/>
-      <c r="U26" s="7" t="n"/>
-      <c r="V26" s="7" t="n"/>
-      <c r="W26" s="7" t="n"/>
-      <c r="X26" s="7" t="n"/>
-      <c r="Y26" s="7" t="n"/>
-      <c r="Z26" s="7" t="n"/>
       <c r="AA26" s="8">
         <f>SUM(C26,I26,O26,U26)-4</f>
         <v/>
@@ -1857,32 +1334,6 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="6" t="n"/>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="7" t="n"/>
-      <c r="D27" s="7" t="n"/>
-      <c r="E27" s="7" t="n"/>
-      <c r="F27" s="7" t="n"/>
-      <c r="G27" s="7" t="n"/>
-      <c r="H27" s="7" t="n"/>
-      <c r="I27" s="7" t="n"/>
-      <c r="J27" s="7" t="n"/>
-      <c r="K27" s="7" t="n"/>
-      <c r="L27" s="7" t="n"/>
-      <c r="M27" s="7" t="n"/>
-      <c r="N27" s="7" t="n"/>
-      <c r="O27" s="7" t="n"/>
-      <c r="P27" s="7" t="n"/>
-      <c r="Q27" s="7" t="n"/>
-      <c r="R27" s="7" t="n"/>
-      <c r="S27" s="7" t="n"/>
-      <c r="T27" s="7" t="n"/>
-      <c r="U27" s="7" t="n"/>
-      <c r="V27" s="7" t="n"/>
-      <c r="W27" s="7" t="n"/>
-      <c r="X27" s="7" t="n"/>
-      <c r="Y27" s="7" t="n"/>
-      <c r="Z27" s="7" t="n"/>
       <c r="AA27" s="8">
         <f>SUM(C27,I27,O27,U27)-4</f>
         <v/>
@@ -1909,32 +1360,6 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="7" t="n"/>
-      <c r="D28" s="7" t="n"/>
-      <c r="E28" s="7" t="n"/>
-      <c r="F28" s="7" t="n"/>
-      <c r="G28" s="7" t="n"/>
-      <c r="H28" s="7" t="n"/>
-      <c r="I28" s="7" t="n"/>
-      <c r="J28" s="7" t="n"/>
-      <c r="K28" s="7" t="n"/>
-      <c r="L28" s="7" t="n"/>
-      <c r="M28" s="7" t="n"/>
-      <c r="N28" s="7" t="n"/>
-      <c r="O28" s="7" t="n"/>
-      <c r="P28" s="7" t="n"/>
-      <c r="Q28" s="7" t="n"/>
-      <c r="R28" s="7" t="n"/>
-      <c r="S28" s="7" t="n"/>
-      <c r="T28" s="7" t="n"/>
-      <c r="U28" s="7" t="n"/>
-      <c r="V28" s="7" t="n"/>
-      <c r="W28" s="7" t="n"/>
-      <c r="X28" s="7" t="n"/>
-      <c r="Y28" s="7" t="n"/>
-      <c r="Z28" s="7" t="n"/>
       <c r="AA28" s="8">
         <f>SUM(C28,I28,O28,U28)-4</f>
         <v/>
@@ -1961,32 +1386,6 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="6" t="n"/>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="7" t="n"/>
-      <c r="D29" s="7" t="n"/>
-      <c r="E29" s="7" t="n"/>
-      <c r="F29" s="7" t="n"/>
-      <c r="G29" s="7" t="n"/>
-      <c r="H29" s="7" t="n"/>
-      <c r="I29" s="7" t="n"/>
-      <c r="J29" s="7" t="n"/>
-      <c r="K29" s="7" t="n"/>
-      <c r="L29" s="7" t="n"/>
-      <c r="M29" s="7" t="n"/>
-      <c r="N29" s="7" t="n"/>
-      <c r="O29" s="7" t="n"/>
-      <c r="P29" s="7" t="n"/>
-      <c r="Q29" s="7" t="n"/>
-      <c r="R29" s="7" t="n"/>
-      <c r="S29" s="7" t="n"/>
-      <c r="T29" s="7" t="n"/>
-      <c r="U29" s="7" t="n"/>
-      <c r="V29" s="7" t="n"/>
-      <c r="W29" s="7" t="n"/>
-      <c r="X29" s="7" t="n"/>
-      <c r="Y29" s="7" t="n"/>
-      <c r="Z29" s="7" t="n"/>
       <c r="AA29" s="8">
         <f>SUM(C29,I29,O29,U29)-4</f>
         <v/>
@@ -2013,32 +1412,6 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="n"/>
-      <c r="C30" s="7" t="n"/>
-      <c r="D30" s="7" t="n"/>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="7" t="n"/>
-      <c r="G30" s="7" t="n"/>
-      <c r="H30" s="7" t="n"/>
-      <c r="I30" s="7" t="n"/>
-      <c r="J30" s="7" t="n"/>
-      <c r="K30" s="7" t="n"/>
-      <c r="L30" s="7" t="n"/>
-      <c r="M30" s="7" t="n"/>
-      <c r="N30" s="7" t="n"/>
-      <c r="O30" s="7" t="n"/>
-      <c r="P30" s="7" t="n"/>
-      <c r="Q30" s="7" t="n"/>
-      <c r="R30" s="7" t="n"/>
-      <c r="S30" s="7" t="n"/>
-      <c r="T30" s="7" t="n"/>
-      <c r="U30" s="7" t="n"/>
-      <c r="V30" s="7" t="n"/>
-      <c r="W30" s="7" t="n"/>
-      <c r="X30" s="7" t="n"/>
-      <c r="Y30" s="7" t="n"/>
-      <c r="Z30" s="7" t="n"/>
       <c r="AA30" s="8">
         <f>SUM(C30,I30,O30,U30)-4</f>
         <v/>
@@ -2065,32 +1438,6 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="6" t="n"/>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="7" t="n"/>
-      <c r="D31" s="7" t="n"/>
-      <c r="E31" s="7" t="n"/>
-      <c r="F31" s="7" t="n"/>
-      <c r="G31" s="7" t="n"/>
-      <c r="H31" s="7" t="n"/>
-      <c r="I31" s="7" t="n"/>
-      <c r="J31" s="7" t="n"/>
-      <c r="K31" s="7" t="n"/>
-      <c r="L31" s="7" t="n"/>
-      <c r="M31" s="7" t="n"/>
-      <c r="N31" s="7" t="n"/>
-      <c r="O31" s="7" t="n"/>
-      <c r="P31" s="7" t="n"/>
-      <c r="Q31" s="7" t="n"/>
-      <c r="R31" s="7" t="n"/>
-      <c r="S31" s="7" t="n"/>
-      <c r="T31" s="7" t="n"/>
-      <c r="U31" s="7" t="n"/>
-      <c r="V31" s="7" t="n"/>
-      <c r="W31" s="7" t="n"/>
-      <c r="X31" s="7" t="n"/>
-      <c r="Y31" s="7" t="n"/>
-      <c r="Z31" s="7" t="n"/>
       <c r="AA31" s="8">
         <f>SUM(C31,I31,O31,U31)-4</f>
         <v/>
@@ -2117,32 +1464,6 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="7" t="n"/>
-      <c r="D32" s="7" t="n"/>
-      <c r="E32" s="7" t="n"/>
-      <c r="F32" s="7" t="n"/>
-      <c r="G32" s="7" t="n"/>
-      <c r="H32" s="7" t="n"/>
-      <c r="I32" s="7" t="n"/>
-      <c r="J32" s="7" t="n"/>
-      <c r="K32" s="7" t="n"/>
-      <c r="L32" s="7" t="n"/>
-      <c r="M32" s="7" t="n"/>
-      <c r="N32" s="7" t="n"/>
-      <c r="O32" s="7" t="n"/>
-      <c r="P32" s="7" t="n"/>
-      <c r="Q32" s="7" t="n"/>
-      <c r="R32" s="7" t="n"/>
-      <c r="S32" s="7" t="n"/>
-      <c r="T32" s="7" t="n"/>
-      <c r="U32" s="7" t="n"/>
-      <c r="V32" s="7" t="n"/>
-      <c r="W32" s="7" t="n"/>
-      <c r="X32" s="7" t="n"/>
-      <c r="Y32" s="7" t="n"/>
-      <c r="Z32" s="7" t="n"/>
       <c r="AA32" s="8">
         <f>SUM(C32,I32,O32,U32)-4</f>
         <v/>
@@ -2169,32 +1490,6 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="6" t="n"/>
-      <c r="B33" s="6" t="n"/>
-      <c r="C33" s="7" t="n"/>
-      <c r="D33" s="7" t="n"/>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="7" t="n"/>
-      <c r="G33" s="7" t="n"/>
-      <c r="H33" s="7" t="n"/>
-      <c r="I33" s="7" t="n"/>
-      <c r="J33" s="7" t="n"/>
-      <c r="K33" s="7" t="n"/>
-      <c r="L33" s="7" t="n"/>
-      <c r="M33" s="7" t="n"/>
-      <c r="N33" s="7" t="n"/>
-      <c r="O33" s="7" t="n"/>
-      <c r="P33" s="7" t="n"/>
-      <c r="Q33" s="7" t="n"/>
-      <c r="R33" s="7" t="n"/>
-      <c r="S33" s="7" t="n"/>
-      <c r="T33" s="7" t="n"/>
-      <c r="U33" s="7" t="n"/>
-      <c r="V33" s="7" t="n"/>
-      <c r="W33" s="7" t="n"/>
-      <c r="X33" s="7" t="n"/>
-      <c r="Y33" s="7" t="n"/>
-      <c r="Z33" s="7" t="n"/>
       <c r="AA33" s="8">
         <f>SUM(C33,I33,O33,U33)-4</f>
         <v/>
@@ -2221,32 +1516,6 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="6" t="n"/>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="7" t="n"/>
-      <c r="D34" s="7" t="n"/>
-      <c r="E34" s="7" t="n"/>
-      <c r="F34" s="7" t="n"/>
-      <c r="G34" s="7" t="n"/>
-      <c r="H34" s="7" t="n"/>
-      <c r="I34" s="7" t="n"/>
-      <c r="J34" s="7" t="n"/>
-      <c r="K34" s="7" t="n"/>
-      <c r="L34" s="7" t="n"/>
-      <c r="M34" s="7" t="n"/>
-      <c r="N34" s="7" t="n"/>
-      <c r="O34" s="7" t="n"/>
-      <c r="P34" s="7" t="n"/>
-      <c r="Q34" s="7" t="n"/>
-      <c r="R34" s="7" t="n"/>
-      <c r="S34" s="7" t="n"/>
-      <c r="T34" s="7" t="n"/>
-      <c r="U34" s="7" t="n"/>
-      <c r="V34" s="7" t="n"/>
-      <c r="W34" s="7" t="n"/>
-      <c r="X34" s="7" t="n"/>
-      <c r="Y34" s="7" t="n"/>
-      <c r="Z34" s="7" t="n"/>
       <c r="AA34" s="8">
         <f>SUM(C34,I34,O34,U34)-4</f>
         <v/>
@@ -2273,32 +1542,6 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="6" t="n"/>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="7" t="n"/>
-      <c r="G35" s="7" t="n"/>
-      <c r="H35" s="7" t="n"/>
-      <c r="I35" s="7" t="n"/>
-      <c r="J35" s="7" t="n"/>
-      <c r="K35" s="7" t="n"/>
-      <c r="L35" s="7" t="n"/>
-      <c r="M35" s="7" t="n"/>
-      <c r="N35" s="7" t="n"/>
-      <c r="O35" s="7" t="n"/>
-      <c r="P35" s="7" t="n"/>
-      <c r="Q35" s="7" t="n"/>
-      <c r="R35" s="7" t="n"/>
-      <c r="S35" s="7" t="n"/>
-      <c r="T35" s="7" t="n"/>
-      <c r="U35" s="7" t="n"/>
-      <c r="V35" s="7" t="n"/>
-      <c r="W35" s="7" t="n"/>
-      <c r="X35" s="7" t="n"/>
-      <c r="Y35" s="7" t="n"/>
-      <c r="Z35" s="7" t="n"/>
       <c r="AA35" s="8">
         <f>SUM(C35,I35,O35,U35)-4</f>
         <v/>
@@ -2325,32 +1568,6 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6" t="n"/>
-      <c r="C36" s="7" t="n"/>
-      <c r="D36" s="7" t="n"/>
-      <c r="E36" s="7" t="n"/>
-      <c r="F36" s="7" t="n"/>
-      <c r="G36" s="7" t="n"/>
-      <c r="H36" s="7" t="n"/>
-      <c r="I36" s="7" t="n"/>
-      <c r="J36" s="7" t="n"/>
-      <c r="K36" s="7" t="n"/>
-      <c r="L36" s="7" t="n"/>
-      <c r="M36" s="7" t="n"/>
-      <c r="N36" s="7" t="n"/>
-      <c r="O36" s="7" t="n"/>
-      <c r="P36" s="7" t="n"/>
-      <c r="Q36" s="7" t="n"/>
-      <c r="R36" s="7" t="n"/>
-      <c r="S36" s="7" t="n"/>
-      <c r="T36" s="7" t="n"/>
-      <c r="U36" s="7" t="n"/>
-      <c r="V36" s="7" t="n"/>
-      <c r="W36" s="7" t="n"/>
-      <c r="X36" s="7" t="n"/>
-      <c r="Y36" s="7" t="n"/>
-      <c r="Z36" s="7" t="n"/>
       <c r="AA36" s="8">
         <f>SUM(C36,I36,O36,U36)-4</f>
         <v/>
@@ -2377,32 +1594,6 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="6" t="n"/>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="7" t="n"/>
-      <c r="D37" s="7" t="n"/>
-      <c r="E37" s="7" t="n"/>
-      <c r="F37" s="7" t="n"/>
-      <c r="G37" s="7" t="n"/>
-      <c r="H37" s="7" t="n"/>
-      <c r="I37" s="7" t="n"/>
-      <c r="J37" s="7" t="n"/>
-      <c r="K37" s="7" t="n"/>
-      <c r="L37" s="7" t="n"/>
-      <c r="M37" s="7" t="n"/>
-      <c r="N37" s="7" t="n"/>
-      <c r="O37" s="7" t="n"/>
-      <c r="P37" s="7" t="n"/>
-      <c r="Q37" s="7" t="n"/>
-      <c r="R37" s="7" t="n"/>
-      <c r="S37" s="7" t="n"/>
-      <c r="T37" s="7" t="n"/>
-      <c r="U37" s="7" t="n"/>
-      <c r="V37" s="7" t="n"/>
-      <c r="W37" s="7" t="n"/>
-      <c r="X37" s="7" t="n"/>
-      <c r="Y37" s="7" t="n"/>
-      <c r="Z37" s="7" t="n"/>
       <c r="AA37" s="8">
         <f>SUM(C37,I37,O37,U37)-4</f>
         <v/>
@@ -2429,32 +1620,6 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6" t="n"/>
-      <c r="C38" s="7" t="n"/>
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
-      <c r="F38" s="7" t="n"/>
-      <c r="G38" s="7" t="n"/>
-      <c r="H38" s="7" t="n"/>
-      <c r="I38" s="7" t="n"/>
-      <c r="J38" s="7" t="n"/>
-      <c r="K38" s="7" t="n"/>
-      <c r="L38" s="7" t="n"/>
-      <c r="M38" s="7" t="n"/>
-      <c r="N38" s="7" t="n"/>
-      <c r="O38" s="7" t="n"/>
-      <c r="P38" s="7" t="n"/>
-      <c r="Q38" s="7" t="n"/>
-      <c r="R38" s="7" t="n"/>
-      <c r="S38" s="7" t="n"/>
-      <c r="T38" s="7" t="n"/>
-      <c r="U38" s="7" t="n"/>
-      <c r="V38" s="7" t="n"/>
-      <c r="W38" s="7" t="n"/>
-      <c r="X38" s="7" t="n"/>
-      <c r="Y38" s="7" t="n"/>
-      <c r="Z38" s="7" t="n"/>
       <c r="AA38" s="8">
         <f>SUM(C38,I38,O38,U38)-4</f>
         <v/>
@@ -2481,32 +1646,6 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="n"/>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="7" t="n"/>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="7" t="n"/>
-      <c r="F39" s="7" t="n"/>
-      <c r="G39" s="7" t="n"/>
-      <c r="H39" s="7" t="n"/>
-      <c r="I39" s="7" t="n"/>
-      <c r="J39" s="7" t="n"/>
-      <c r="K39" s="7" t="n"/>
-      <c r="L39" s="7" t="n"/>
-      <c r="M39" s="7" t="n"/>
-      <c r="N39" s="7" t="n"/>
-      <c r="O39" s="7" t="n"/>
-      <c r="P39" s="7" t="n"/>
-      <c r="Q39" s="7" t="n"/>
-      <c r="R39" s="7" t="n"/>
-      <c r="S39" s="7" t="n"/>
-      <c r="T39" s="7" t="n"/>
-      <c r="U39" s="7" t="n"/>
-      <c r="V39" s="7" t="n"/>
-      <c r="W39" s="7" t="n"/>
-      <c r="X39" s="7" t="n"/>
-      <c r="Y39" s="7" t="n"/>
-      <c r="Z39" s="7" t="n"/>
       <c r="AA39" s="8">
         <f>SUM(C39,I39,O39,U39)-4</f>
         <v/>
@@ -2533,32 +1672,6 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="6" t="n"/>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="7" t="n"/>
-      <c r="D40" s="7" t="n"/>
-      <c r="E40" s="7" t="n"/>
-      <c r="F40" s="7" t="n"/>
-      <c r="G40" s="7" t="n"/>
-      <c r="H40" s="7" t="n"/>
-      <c r="I40" s="7" t="n"/>
-      <c r="J40" s="7" t="n"/>
-      <c r="K40" s="7" t="n"/>
-      <c r="L40" s="7" t="n"/>
-      <c r="M40" s="7" t="n"/>
-      <c r="N40" s="7" t="n"/>
-      <c r="O40" s="7" t="n"/>
-      <c r="P40" s="7" t="n"/>
-      <c r="Q40" s="7" t="n"/>
-      <c r="R40" s="7" t="n"/>
-      <c r="S40" s="7" t="n"/>
-      <c r="T40" s="7" t="n"/>
-      <c r="U40" s="7" t="n"/>
-      <c r="V40" s="7" t="n"/>
-      <c r="W40" s="7" t="n"/>
-      <c r="X40" s="7" t="n"/>
-      <c r="Y40" s="7" t="n"/>
-      <c r="Z40" s="7" t="n"/>
       <c r="AA40" s="8">
         <f>SUM(C40,I40,O40,U40)-4</f>
         <v/>
@@ -2585,32 +1698,6 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="6" t="n"/>
-      <c r="B41" s="6" t="n"/>
-      <c r="C41" s="7" t="n"/>
-      <c r="D41" s="7" t="n"/>
-      <c r="E41" s="7" t="n"/>
-      <c r="F41" s="7" t="n"/>
-      <c r="G41" s="7" t="n"/>
-      <c r="H41" s="7" t="n"/>
-      <c r="I41" s="7" t="n"/>
-      <c r="J41" s="7" t="n"/>
-      <c r="K41" s="7" t="n"/>
-      <c r="L41" s="7" t="n"/>
-      <c r="M41" s="7" t="n"/>
-      <c r="N41" s="7" t="n"/>
-      <c r="O41" s="7" t="n"/>
-      <c r="P41" s="7" t="n"/>
-      <c r="Q41" s="7" t="n"/>
-      <c r="R41" s="7" t="n"/>
-      <c r="S41" s="7" t="n"/>
-      <c r="T41" s="7" t="n"/>
-      <c r="U41" s="7" t="n"/>
-      <c r="V41" s="7" t="n"/>
-      <c r="W41" s="7" t="n"/>
-      <c r="X41" s="7" t="n"/>
-      <c r="Y41" s="7" t="n"/>
-      <c r="Z41" s="7" t="n"/>
       <c r="AA41" s="8">
         <f>SUM(C41,I41,O41,U41)-4</f>
         <v/>
@@ -2637,32 +1724,6 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="6" t="n"/>
-      <c r="B42" s="6" t="n"/>
-      <c r="C42" s="7" t="n"/>
-      <c r="D42" s="7" t="n"/>
-      <c r="E42" s="7" t="n"/>
-      <c r="F42" s="7" t="n"/>
-      <c r="G42" s="7" t="n"/>
-      <c r="H42" s="7" t="n"/>
-      <c r="I42" s="7" t="n"/>
-      <c r="J42" s="7" t="n"/>
-      <c r="K42" s="7" t="n"/>
-      <c r="L42" s="7" t="n"/>
-      <c r="M42" s="7" t="n"/>
-      <c r="N42" s="7" t="n"/>
-      <c r="O42" s="7" t="n"/>
-      <c r="P42" s="7" t="n"/>
-      <c r="Q42" s="7" t="n"/>
-      <c r="R42" s="7" t="n"/>
-      <c r="S42" s="7" t="n"/>
-      <c r="T42" s="7" t="n"/>
-      <c r="U42" s="7" t="n"/>
-      <c r="V42" s="7" t="n"/>
-      <c r="W42" s="7" t="n"/>
-      <c r="X42" s="7" t="n"/>
-      <c r="Y42" s="7" t="n"/>
-      <c r="Z42" s="7" t="n"/>
       <c r="AA42" s="8">
         <f>SUM(C42,I42,O42,U42)-4</f>
         <v/>
@@ -2689,32 +1750,6 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="6" t="n"/>
-      <c r="B43" s="6" t="n"/>
-      <c r="C43" s="7" t="n"/>
-      <c r="D43" s="7" t="n"/>
-      <c r="E43" s="7" t="n"/>
-      <c r="F43" s="7" t="n"/>
-      <c r="G43" s="7" t="n"/>
-      <c r="H43" s="7" t="n"/>
-      <c r="I43" s="7" t="n"/>
-      <c r="J43" s="7" t="n"/>
-      <c r="K43" s="7" t="n"/>
-      <c r="L43" s="7" t="n"/>
-      <c r="M43" s="7" t="n"/>
-      <c r="N43" s="7" t="n"/>
-      <c r="O43" s="7" t="n"/>
-      <c r="P43" s="7" t="n"/>
-      <c r="Q43" s="7" t="n"/>
-      <c r="R43" s="7" t="n"/>
-      <c r="S43" s="7" t="n"/>
-      <c r="T43" s="7" t="n"/>
-      <c r="U43" s="7" t="n"/>
-      <c r="V43" s="7" t="n"/>
-      <c r="W43" s="7" t="n"/>
-      <c r="X43" s="7" t="n"/>
-      <c r="Y43" s="7" t="n"/>
-      <c r="Z43" s="7" t="n"/>
       <c r="AA43" s="8">
         <f>SUM(C43,I43,O43,U43)-4</f>
         <v/>
@@ -2741,32 +1776,6 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="6" t="n"/>
-      <c r="B44" s="6" t="n"/>
-      <c r="C44" s="7" t="n"/>
-      <c r="D44" s="7" t="n"/>
-      <c r="E44" s="7" t="n"/>
-      <c r="F44" s="7" t="n"/>
-      <c r="G44" s="7" t="n"/>
-      <c r="H44" s="7" t="n"/>
-      <c r="I44" s="7" t="n"/>
-      <c r="J44" s="7" t="n"/>
-      <c r="K44" s="7" t="n"/>
-      <c r="L44" s="7" t="n"/>
-      <c r="M44" s="7" t="n"/>
-      <c r="N44" s="7" t="n"/>
-      <c r="O44" s="7" t="n"/>
-      <c r="P44" s="7" t="n"/>
-      <c r="Q44" s="7" t="n"/>
-      <c r="R44" s="7" t="n"/>
-      <c r="S44" s="7" t="n"/>
-      <c r="T44" s="7" t="n"/>
-      <c r="U44" s="7" t="n"/>
-      <c r="V44" s="7" t="n"/>
-      <c r="W44" s="7" t="n"/>
-      <c r="X44" s="7" t="n"/>
-      <c r="Y44" s="7" t="n"/>
-      <c r="Z44" s="7" t="n"/>
       <c r="AA44" s="8">
         <f>SUM(C44,I44,O44,U44)-4</f>
         <v/>
@@ -2793,32 +1802,6 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="6" t="n"/>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
-      <c r="E45" s="7" t="n"/>
-      <c r="F45" s="7" t="n"/>
-      <c r="G45" s="7" t="n"/>
-      <c r="H45" s="7" t="n"/>
-      <c r="I45" s="7" t="n"/>
-      <c r="J45" s="7" t="n"/>
-      <c r="K45" s="7" t="n"/>
-      <c r="L45" s="7" t="n"/>
-      <c r="M45" s="7" t="n"/>
-      <c r="N45" s="7" t="n"/>
-      <c r="O45" s="7" t="n"/>
-      <c r="P45" s="7" t="n"/>
-      <c r="Q45" s="7" t="n"/>
-      <c r="R45" s="7" t="n"/>
-      <c r="S45" s="7" t="n"/>
-      <c r="T45" s="7" t="n"/>
-      <c r="U45" s="7" t="n"/>
-      <c r="V45" s="7" t="n"/>
-      <c r="W45" s="7" t="n"/>
-      <c r="X45" s="7" t="n"/>
-      <c r="Y45" s="7" t="n"/>
-      <c r="Z45" s="7" t="n"/>
       <c r="AA45" s="8">
         <f>SUM(C45,I45,O45,U45)-4</f>
         <v/>
@@ -2845,32 +1828,6 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="6" t="n"/>
-      <c r="B46" s="6" t="n"/>
-      <c r="C46" s="7" t="n"/>
-      <c r="D46" s="7" t="n"/>
-      <c r="E46" s="7" t="n"/>
-      <c r="F46" s="7" t="n"/>
-      <c r="G46" s="7" t="n"/>
-      <c r="H46" s="7" t="n"/>
-      <c r="I46" s="7" t="n"/>
-      <c r="J46" s="7" t="n"/>
-      <c r="K46" s="7" t="n"/>
-      <c r="L46" s="7" t="n"/>
-      <c r="M46" s="7" t="n"/>
-      <c r="N46" s="7" t="n"/>
-      <c r="O46" s="7" t="n"/>
-      <c r="P46" s="7" t="n"/>
-      <c r="Q46" s="7" t="n"/>
-      <c r="R46" s="7" t="n"/>
-      <c r="S46" s="7" t="n"/>
-      <c r="T46" s="7" t="n"/>
-      <c r="U46" s="7" t="n"/>
-      <c r="V46" s="7" t="n"/>
-      <c r="W46" s="7" t="n"/>
-      <c r="X46" s="7" t="n"/>
-      <c r="Y46" s="7" t="n"/>
-      <c r="Z46" s="7" t="n"/>
       <c r="AA46" s="8">
         <f>SUM(C46,I46,O46,U46)-4</f>
         <v/>
@@ -2896,17 +1853,43 @@
         <v/>
       </c>
     </row>
+    <row r="47">
+      <c r="AA47" s="8">
+        <f>SUM(C47,I47,O47,U47)-4</f>
+        <v/>
+      </c>
+      <c r="AB47" s="8">
+        <f>SUM(D47,J47,P47,V47)-4</f>
+        <v/>
+      </c>
+      <c r="AC47" s="8">
+        <f>SUM(E47,K47,Q47,W47)-4</f>
+        <v/>
+      </c>
+      <c r="AD47" s="8">
+        <f>SUM(F47,L47,R47,X47)-4</f>
+        <v/>
+      </c>
+      <c r="AE47" s="8">
+        <f>SUM(G47,M47,S47,Y47)-4</f>
+        <v/>
+      </c>
+      <c r="AF47" s="8">
+        <f>SUM(H47,N47,T47,Z47)-4</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:AF1"/>
+    <mergeCell ref="B4:E4"/>
     <mergeCell ref="A2:AF3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="C6:Z46" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor inválido" error="Solo se permiten los valores 0, 1 o 2." type="list">
+    <dataValidation sqref="C7:Z47" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor no válido" error="La respuesta debe ser 1, 2 o 3." type="list">
       <formula1>"1,2,3"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Colegio/Curso opcionales en el Excel; si faltan, se preguntan al subir el archivo
</commit_message>
<xml_diff>
--- a/assets/Planilla_de_correccion.xlsx
+++ b/assets/Planilla_de_correccion.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,10 @@
     <font>
       <b val="1"/>
       <color rgb="00402A63"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="002B2140"/>
       <sz val="11"/>
     </font>
     <font>
@@ -92,16 +96,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C9BEDD"/>
+        <color rgb="008A6BC0"/>
       </left>
       <right style="thin">
-        <color rgb="00C9BEDD"/>
+        <color rgb="008A6BC0"/>
       </right>
       <top style="thin">
-        <color rgb="00C9BEDD"/>
+        <color rgb="008A6BC0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C9BEDD"/>
+        <color rgb="008A6BC0"/>
       </bottom>
     </border>
   </borders>
@@ -116,16 +120,18 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -497,7 +503,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
     <col width="4.5" customWidth="1" min="3" max="3"/>
     <col width="4.5" customWidth="1" min="4" max="4"/>
     <col width="4.5" customWidth="1" min="5" max="5"/>
@@ -540,33 +546,30 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Completa una fila por estudiante: Nombre, RUT (opcional — muchos estudiantes de esta edad no lo saben de memoria) y las 24 respuestas en el mismo orden en que aparecen en la hoja de aplicación en papel (3 = Me gusta/Me interesa · 2 = No sé · 1 = No me gusta/No me interesa). Las columnas de área (fondo gris, en negrita) se calculan solas — no las edites. Completa Colegio, Curso y Letra UNA SOLA VEZ en los campos de abajo: valen para todos los estudiantes de este archivo (cada planilla es siempre un curso de un colegio). Cuando termines, sube este mismo archivo .xlsx directamente en la app, en la pestaña "Ingresar datos".</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="46" customHeight="1"/>
+          <t>Completa una fila por estudiante: Nombre, RUT (opcional — muchos estudiantes de esta edad no lo saben de memoria) y las 24 respuestas en el mismo orden en que aparecen en la hoja de aplicación en papel (3 = Me gusta/Me interesa · 2 = No sé · 1 = No me gusta/No me interesa). Las columnas de área (fondo gris, en negrita) se calculan solas — no las edites. El Colegio y el Curso son OPCIONALES aquí abajo (celdas B4 y D4): si los completas, valen para todos los estudiantes de este archivo; si los dejas en blanco, la app te los va a preguntar al momento de subir el archivo. Cuando termines, sube este mismo archivo .xlsx directamente en la app, en la pestaña "Ingresar datos".</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="44" customHeight="1"/>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Colegio:</t>
+          <t>Colegio (opcional):</t>
         </is>
       </c>
       <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Curso (opcional):</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>Curso:</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Letra:</t>
         </is>
       </c>
-      <c r="I4" s="4" t="n"/>
+      <c r="F4" s="4" t="n"/>
     </row>
     <row r="5" ht="6" customHeight="1"/>
     <row r="6" ht="32" customHeight="1">
@@ -1880,9 +1883,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:AF1"/>
-    <mergeCell ref="B4:E4"/>
     <mergeCell ref="A2:AF3"/>
   </mergeCells>
   <dataValidations count="1">

</xml_diff>